<commit_message>
Daily NSE scan: 2026-10-01
</commit_message>
<xml_diff>
--- a/output/2026-10-01/enriched_analysis.xlsx
+++ b/output/2026-10-01/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.664</v>
+        <v>2.702</v>
       </c>
       <c r="W2" t="n">
-        <v>2928</v>
+        <v>2886</v>
       </c>
       <c r="X2" t="n">
-        <v>22.9</v>
+        <v>22.6</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.533</v>
+        <v>0.537</v>
       </c>
       <c r="W3" t="n">
-        <v>926</v>
+        <v>920</v>
       </c>
       <c r="X3" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y3" t="n">
         <v>47</v>
@@ -1396,10 +1396,10 @@
         <v>0.049</v>
       </c>
       <c r="W4" t="n">
-        <v>2729</v>
+        <v>2721</v>
       </c>
       <c r="X4" t="n">
-        <v>9.380000000000001</v>
+        <v>9.33</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.952</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="X5" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="Y5" t="n">
         <v>22</v>
@@ -1857,13 +1857,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.316</v>
+        <v>0.321</v>
       </c>
       <c r="W6" t="n">
-        <v>968</v>
+        <v>955</v>
       </c>
       <c r="X6" t="n">
-        <v>9.52</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="Y6" t="n">
         <v>7</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.993</v>
+        <v>0.979</v>
       </c>
       <c r="W7" t="n">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="X7" t="n">
-        <v>8.6</v>
+        <v>8.73</v>
       </c>
       <c r="Y7" t="n">
         <v>17</v>
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>2.212</v>
+        <v>2.262</v>
       </c>
       <c r="W8" t="n">
-        <v>2653</v>
+        <v>2595</v>
       </c>
       <c r="X8" t="n">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="Y8" t="n">
         <v>6</v>
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.472</v>
+        <v>0.48</v>
       </c>
       <c r="W9" t="n">
-        <v>2753</v>
+        <v>2704</v>
       </c>
       <c r="X9" t="n">
-        <v>22.6</v>
+        <v>22.2</v>
       </c>
       <c r="Y9" t="n">
         <v>8</v>
@@ -2713,12 +2713,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2730,40 +2730,40 @@
         </is>
       </c>
       <c r="E10" t="n">
+        <v>19</v>
+      </c>
+      <c r="F10" t="n">
         <v>5</v>
       </c>
-      <c r="F10" t="n">
-        <v>22</v>
-      </c>
       <c r="G10" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>68.59999999999999</v>
+        <v>1043.35</v>
       </c>
       <c r="J10" t="n">
-        <v>64.48999999999999</v>
+        <v>799.34</v>
       </c>
       <c r="K10" t="n">
-        <v>6.4</v>
+        <v>30.5</v>
       </c>
       <c r="L10" t="n">
-        <v>64.29000000000001</v>
+        <v>61.71</v>
       </c>
       <c r="M10" t="n">
-        <v>0.57</v>
+        <v>3.2</v>
       </c>
       <c r="N10" t="n">
-        <v>5656038</v>
+        <v>32023110</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>5656038</v>
+        <v>32023110</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -2777,62 +2777,62 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
+        <v>8</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="W10" t="n">
+        <v>316</v>
+      </c>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="n">
         <v>9</v>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>18-09-2026</t>
-        </is>
-      </c>
-      <c r="V10" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="W10" t="n">
-        <v>843</v>
-      </c>
-      <c r="X10" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>19</v>
-      </c>
       <c r="Z10" t="n">
-        <v>12.31</v>
+        <v>11.91</v>
       </c>
       <c r="AA10" t="n">
-        <v>41</v>
+        <v>-184</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.8</v>
+        <v>31.98</v>
       </c>
       <c r="AC10" t="n">
-        <v>22.2</v>
+        <v>-0.26</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="AE10" t="b">
         <v>1</v>
       </c>
       <c r="AF10" t="n">
-        <v>12.14</v>
+        <v>57.93</v>
       </c>
       <c r="AG10" t="n">
-        <v>66.02</v>
-      </c>
-      <c r="AH10" t="inlineStr"/>
+        <v>816.35</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>787.17</v>
+      </c>
       <c r="AI10" t="n">
-        <v>35.4</v>
+        <v>28.8</v>
       </c>
       <c r="AJ10" t="n">
-        <v>64.49302166476625</v>
+        <v>799.3387748989066</v>
       </c>
       <c r="AK10" t="n">
-        <v>6.4</v>
+        <v>30.5</v>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AN10" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO10" t="inlineStr">
@@ -2852,47 +2852,47 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>28-09-2026</t>
         </is>
       </c>
       <c r="AQ10" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="AR10" t="n">
         <v>45</v>
       </c>
       <c r="AS10" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU10" t="n">
         <v>4</v>
       </c>
       <c r="AV10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AW10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AX10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AY10" t="n">
-        <v>0</v>
+        <v>3257615</v>
       </c>
       <c r="AZ10" t="n">
-        <v>1628129</v>
+        <v>10731521</v>
       </c>
       <c r="BA10" t="n">
-        <v>2601121</v>
+        <v>15906207</v>
       </c>
       <c r="BB10" t="n">
-        <v>5656038</v>
+        <v>32023110</v>
       </c>
       <c r="BC10" t="n">
-        <v>5656038</v>
+        <v>32023110</v>
       </c>
       <c r="BD10" t="n">
         <v>0</v>
@@ -2925,34 +2925,34 @@
         <v>0</v>
       </c>
       <c r="BN10" t="n">
-        <v>0</v>
+        <v>3257615</v>
       </c>
       <c r="BO10" t="n">
-        <v>2601121</v>
+        <v>15906207</v>
       </c>
       <c r="BP10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BQ10" t="n">
         <v>0</v>
       </c>
       <c r="BR10" t="n">
-        <v>0</v>
+        <v>0.2048</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2960,40 +2960,40 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G11" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>5062</v>
+        <v>140.49</v>
       </c>
       <c r="J11" t="n">
-        <v>5198.76</v>
+        <v>171.54</v>
       </c>
       <c r="K11" t="n">
-        <v>-2.6</v>
+        <v>-18.1</v>
       </c>
       <c r="L11" t="n">
-        <v>67.16</v>
+        <v>74.59</v>
       </c>
       <c r="M11" t="n">
-        <v>7.21</v>
+        <v>1.11</v>
       </c>
       <c r="N11" t="n">
-        <v>72054758</v>
+        <v>11081344</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>72054758</v>
+        <v>11081344</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -3007,124 +3007,124 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.046</v>
+        <v>0.063</v>
       </c>
       <c r="W11" t="n">
-        <v>15734</v>
+        <v>1761</v>
       </c>
       <c r="X11" t="n">
-        <v>40.1</v>
+        <v>40.4</v>
       </c>
       <c r="Y11" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA11" t="n">
         <v>83</v>
       </c>
-      <c r="Z11" t="n">
-        <v>145</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>264</v>
-      </c>
       <c r="AB11" t="n">
-        <v>27.38</v>
+        <v>0.8</v>
       </c>
       <c r="AC11" t="n">
-        <v>25.5</v>
+        <v>30.3</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.64</v>
+        <v>0.2</v>
       </c>
       <c r="AE11" t="b">
         <v>1</v>
       </c>
       <c r="AF11" t="n">
+        <v>23</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>178.38</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>487.24</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>171.5378328173375</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>-18.1</v>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>25-08-2026</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ11" t="n">
+        <v>36</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>37</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW11" t="n">
         <v>5</v>
       </c>
-      <c r="AG11" t="n">
-        <v>5436.1</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>4485.08</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>5198.755988455989</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="AL11" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>04-08-2026</t>
-        </is>
-      </c>
-      <c r="AP11" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="AQ11" t="n">
-        <v>27</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>58</v>
-      </c>
-      <c r="AS11" t="n">
-        <v>31</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW11" t="n">
-        <v>6</v>
-      </c>
       <c r="AX11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AY11" t="n">
-        <v>0</v>
+        <v>83720</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0</v>
+        <v>83720</v>
       </c>
       <c r="BA11" t="n">
-        <v>0</v>
+        <v>6160489</v>
       </c>
       <c r="BB11" t="n">
-        <v>72054758</v>
+        <v>11081344</v>
       </c>
       <c r="BC11" t="n">
-        <v>72054758</v>
+        <v>11081344</v>
       </c>
       <c r="BD11" t="n">
         <v>0</v>
@@ -3157,34 +3157,34 @@
         <v>0</v>
       </c>
       <c r="BN11" t="n">
-        <v>0</v>
+        <v>83720</v>
       </c>
       <c r="BO11" t="n">
-        <v>0</v>
+        <v>6160489</v>
       </c>
       <c r="BP11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BQ11" t="n">
         <v>0</v>
       </c>
       <c r="BR11" t="n">
-        <v>0</v>
+        <v>0.0136</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -3192,40 +3192,40 @@
         </is>
       </c>
       <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" t="n">
         <v>17</v>
       </c>
-      <c r="F12" t="n">
-        <v>5</v>
-      </c>
-      <c r="G12" t="n">
-        <v>25</v>
-      </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>1043.35</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>799.34</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>30.5</v>
+        <v>6.4</v>
       </c>
       <c r="L12" t="n">
-        <v>61.71</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>3.2</v>
+        <v>0.57</v>
       </c>
       <c r="N12" t="n">
-        <v>32023110</v>
+        <v>5656038</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>32023110</v>
+        <v>5656038</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -3239,62 +3239,62 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>28-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.991</v>
+        <v>0.065</v>
       </c>
       <c r="W12" t="n">
-        <v>323</v>
-      </c>
-      <c r="X12" t="inlineStr"/>
+        <v>871</v>
+      </c>
+      <c r="X12" t="n">
+        <v>22</v>
+      </c>
       <c r="Y12" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="Z12" t="n">
-        <v>11.91</v>
+        <v>12.31</v>
       </c>
       <c r="AA12" t="n">
-        <v>-184</v>
+        <v>41</v>
       </c>
       <c r="AB12" t="n">
-        <v>31.98</v>
+        <v>0.8</v>
       </c>
       <c r="AC12" t="n">
-        <v>-0.26</v>
+        <v>22.2</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="AE12" t="b">
         <v>1</v>
       </c>
       <c r="AF12" t="n">
-        <v>57.93</v>
+        <v>12.14</v>
       </c>
       <c r="AG12" t="n">
-        <v>816.35</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>787.17</v>
-      </c>
+        <v>66.02</v>
+      </c>
+      <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="n">
-        <v>28.8</v>
+        <v>35.4</v>
       </c>
       <c r="AJ12" t="n">
-        <v>799.3387748989066</v>
+        <v>64.49302166476625</v>
       </c>
       <c r="AK12" t="n">
-        <v>30.5</v>
+        <v>6.4</v>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO12" t="inlineStr">
@@ -3314,47 +3314,47 @@
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>28-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="AQ12" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AR12" t="n">
         <v>45</v>
       </c>
       <c r="AS12" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="AT12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU12" t="n">
         <v>4</v>
       </c>
       <c r="AV12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AX12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AY12" t="n">
-        <v>3257615</v>
+        <v>0</v>
       </c>
       <c r="AZ12" t="n">
-        <v>10731521</v>
+        <v>1628129</v>
       </c>
       <c r="BA12" t="n">
-        <v>15906207</v>
+        <v>2601121</v>
       </c>
       <c r="BB12" t="n">
-        <v>32023110</v>
+        <v>5656038</v>
       </c>
       <c r="BC12" t="n">
-        <v>32023110</v>
+        <v>5656038</v>
       </c>
       <c r="BD12" t="n">
         <v>0</v>
@@ -3387,34 +3387,34 @@
         <v>0</v>
       </c>
       <c r="BN12" t="n">
-        <v>3257615</v>
+        <v>0</v>
       </c>
       <c r="BO12" t="n">
-        <v>15906207</v>
+        <v>2601121</v>
       </c>
       <c r="BP12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BQ12" t="n">
         <v>0</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.2048</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hy-Tech Engineers Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -3422,40 +3422,40 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>72.29000000000001</v>
+        <v>5062</v>
       </c>
       <c r="J13" t="n">
-        <v>68.68000000000001</v>
+        <v>5198.76</v>
       </c>
       <c r="K13" t="n">
-        <v>5.3</v>
+        <v>-2.6</v>
       </c>
       <c r="L13" t="n">
-        <v>71.22</v>
+        <v>67.16</v>
       </c>
       <c r="M13" t="n">
-        <v>0.86</v>
+        <v>7.21</v>
       </c>
       <c r="N13" t="n">
-        <v>8585000</v>
+        <v>72054758</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>8585000</v>
+        <v>72054758</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -3469,118 +3469,124 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.125</v>
+        <v>0.047</v>
       </c>
       <c r="W13" t="n">
-        <v>686</v>
+        <v>15396</v>
       </c>
       <c r="X13" t="n">
-        <v>29.9</v>
+        <v>39.2</v>
       </c>
       <c r="Y13" t="n">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="Z13" t="n">
-        <v>8.44</v>
+        <v>145</v>
       </c>
       <c r="AA13" t="n">
-        <v>39</v>
+        <v>264</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.55</v>
+        <v>27.38</v>
       </c>
       <c r="AC13" t="n">
-        <v>23.9</v>
+        <v>25.5</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.25</v>
+        <v>0.64</v>
       </c>
       <c r="AE13" t="b">
         <v>1</v>
       </c>
       <c r="AF13" t="n">
-        <v>19.61</v>
-      </c>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>5436.1</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>4485.08</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>47.5</v>
+      </c>
       <c r="AJ13" t="n">
-        <v>68.68000000000001</v>
+        <v>5198.755988455989</v>
       </c>
       <c r="AK13" t="n">
-        <v>5.3</v>
+        <v>-2.6</v>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="AQ13" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="AR13" t="n">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="AS13" t="n">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="AT13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AX13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AY13" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="AZ13" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="BA13" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="BB13" t="n">
-        <v>8585000</v>
+        <v>72054758</v>
       </c>
       <c r="BC13" t="n">
-        <v>8585000</v>
+        <v>72054758</v>
       </c>
       <c r="BD13" t="n">
         <v>0</v>
@@ -3613,34 +3619,34 @@
         <v>0</v>
       </c>
       <c r="BN13" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="BO13" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="BP13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ13" t="n">
         <v>0</v>
       </c>
       <c r="BR13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bhageria Industries Limited</t>
+          <t>Hy-Tech Engineers Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -3648,40 +3654,40 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>22</v>
       </c>
       <c r="G14" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>406.45</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>217.8</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>86.59999999999999</v>
+        <v>5.3</v>
       </c>
       <c r="L14" t="n">
-        <v>71.75</v>
+        <v>71.22</v>
       </c>
       <c r="M14" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="N14" t="n">
-        <v>8227124</v>
+        <v>8585000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>8227124</v>
+        <v>8585000</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -3695,124 +3701,118 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.046</v>
+        <v>0.124</v>
       </c>
       <c r="W14" t="n">
-        <v>1774</v>
+        <v>691</v>
       </c>
       <c r="X14" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>39</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AC14" t="n">
         <v>23.9</v>
       </c>
-      <c r="Y14" t="n">
-        <v>55</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>40</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>54</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>8.23</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>11</v>
-      </c>
       <c r="AD14" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="AE14" t="b">
         <v>1</v>
       </c>
       <c r="AF14" t="n">
-        <v>14</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>263.59</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>196.11</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>203.2</v>
-      </c>
+        <v>19.61</v>
+      </c>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="n">
-        <v>217.7985916238683</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="AK14" t="n">
-        <v>86.59999999999999</v>
+        <v>5.3</v>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="AQ14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR14" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="AS14" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="AT14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AX14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AY14" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="BA14" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="BB14" t="n">
-        <v>8227124</v>
+        <v>8585000</v>
       </c>
       <c r="BC14" t="n">
-        <v>8227124</v>
+        <v>8585000</v>
       </c>
       <c r="BD14" t="n">
         <v>0</v>
@@ -3845,10 +3845,10 @@
         <v>0</v>
       </c>
       <c r="BN14" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="BO14" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="BP14" t="n">
         <v>1</v>
@@ -3857,22 +3857,22 @@
         <v>0</v>
       </c>
       <c r="BR14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INDO RAMA SYNTHETICS (INDIA) LIMITED</t>
+          <t>Bhageria Industries Limited</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3880,10 +3880,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G15" t="n">
         <v>25</v>
@@ -3892,28 +3892,28 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>100.36</v>
+        <v>406.45</v>
       </c>
       <c r="J15" t="n">
-        <v>75.68000000000001</v>
+        <v>217.8</v>
       </c>
       <c r="K15" t="n">
-        <v>32.6</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>74.84999999999999</v>
+        <v>71.75</v>
       </c>
       <c r="M15" t="n">
-        <v>3.14</v>
+        <v>0.82</v>
       </c>
       <c r="N15" t="n">
-        <v>31393588</v>
+        <v>8227124</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>31393588</v>
+        <v>8227124</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -3927,69 +3927,69 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>0.12</v>
+        <v>0.049</v>
       </c>
       <c r="W15" t="n">
-        <v>2621</v>
+        <v>1691</v>
       </c>
       <c r="X15" t="n">
-        <v>23</v>
+        <v>22.8</v>
       </c>
       <c r="Y15" t="n">
-        <v>-3</v>
+        <v>55</v>
       </c>
       <c r="Z15" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="AA15" t="n">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.29</v>
+        <v>8.23</v>
       </c>
       <c r="AC15" t="n">
-        <v>15.8</v>
+        <v>11</v>
       </c>
       <c r="AD15" t="n">
-        <v>1.69</v>
+        <v>0.01</v>
       </c>
       <c r="AE15" t="b">
         <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="AG15" t="n">
-        <v>70.39</v>
+        <v>263.59</v>
       </c>
       <c r="AH15" t="n">
-        <v>48.47</v>
+        <v>196.11</v>
       </c>
       <c r="AI15" t="n">
-        <v>223.4</v>
+        <v>203.2</v>
       </c>
       <c r="AJ15" t="n">
-        <v>75.6844038997483</v>
+        <v>217.7985916238683</v>
       </c>
       <c r="AK15" t="n">
-        <v>32.6</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM15" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN15" t="inlineStr">
@@ -3999,22 +3999,22 @@
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="AQ15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR15" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="AS15" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
@@ -4023,13 +4023,13 @@
         <v>0</v>
       </c>
       <c r="AV15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AX15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AY15" t="n">
         <v>0</v>
@@ -4038,13 +4038,13 @@
         <v>0</v>
       </c>
       <c r="BA15" t="n">
-        <v>31393588</v>
+        <v>0</v>
       </c>
       <c r="BB15" t="n">
-        <v>31393588</v>
+        <v>8227124</v>
       </c>
       <c r="BC15" t="n">
-        <v>31393588</v>
+        <v>8227124</v>
       </c>
       <c r="BD15" t="n">
         <v>0</v>
@@ -4080,7 +4080,7 @@
         <v>0</v>
       </c>
       <c r="BO15" t="n">
-        <v>31393588</v>
+        <v>0</v>
       </c>
       <c r="BP15" t="n">
         <v>1</v>
@@ -4095,16 +4095,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VEEGALAND</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>INDO RAMA SYNTHETICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4112,40 +4112,40 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>142.41</v>
+        <v>100.36</v>
       </c>
       <c r="J16" t="n">
-        <v>143.72</v>
+        <v>75.68000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.9</v>
+        <v>32.6</v>
       </c>
       <c r="L16" t="n">
-        <v>63.69</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>19.68</v>
+        <v>3.14</v>
       </c>
       <c r="N16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
@@ -4159,54 +4159,60 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>22-09-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>2.835</v>
+        <v>0.128</v>
       </c>
       <c r="W16" t="n">
-        <v>694</v>
+        <v>2462</v>
       </c>
       <c r="X16" t="n">
-        <v>26.1</v>
+        <v>21.6</v>
       </c>
       <c r="Y16" t="n">
-        <v>30</v>
+        <v>-3</v>
       </c>
       <c r="Z16" t="n">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="AA16" t="n">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="AB16" t="n">
-        <v>7.88</v>
+        <v>1.29</v>
       </c>
       <c r="AC16" t="n">
-        <v>14.1</v>
+        <v>15.8</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.32</v>
+        <v>1.69</v>
       </c>
       <c r="AE16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>16</v>
-      </c>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>70.39</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>48.47</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>223.4</v>
+      </c>
       <c r="AJ16" t="n">
-        <v>143.7164139971926</v>
+        <v>75.6844038997483</v>
       </c>
       <c r="AK16" t="n">
-        <v>-0.9</v>
+        <v>32.6</v>
       </c>
       <c r="AL16" t="inlineStr">
         <is>
@@ -4220,57 +4226,57 @@
       </c>
       <c r="AN16" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>22-09-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="AQ16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AS16" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="AT16" t="n">
         <v>0</v>
       </c>
       <c r="AU16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AW16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AX16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY16" t="n">
         <v>0</v>
       </c>
       <c r="AZ16" t="n">
-        <v>196783125</v>
+        <v>0</v>
       </c>
       <c r="BA16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="BB16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="BC16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="BD16" t="n">
         <v>0</v>
@@ -4306,7 +4312,7 @@
         <v>0</v>
       </c>
       <c r="BO16" t="n">
-        <v>196783125</v>
+        <v>31393588</v>
       </c>
       <c r="BP16" t="n">
         <v>1</v>
@@ -4330,7 +4336,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4338,7 +4344,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
         <v>8</v>
@@ -4393,13 +4399,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.495</v>
+        <v>0.503</v>
       </c>
       <c r="W17" t="n">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="X17" t="n">
-        <v>37.4</v>
+        <v>36.8</v>
       </c>
       <c r="Y17" t="n">
         <v>21</v>
@@ -4553,57 +4559,57 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>VEEGALAND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Avoid</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F18" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>140.49</v>
+        <v>142.41</v>
       </c>
       <c r="J18" t="n">
-        <v>171.84</v>
+        <v>143.72</v>
       </c>
       <c r="K18" t="n">
-        <v>-18.2</v>
+        <v>-0.9</v>
       </c>
       <c r="L18" t="n">
-        <v>74.59</v>
+        <v>63.69</v>
       </c>
       <c r="M18" t="n">
-        <v>1.1</v>
+        <v>19.68</v>
       </c>
       <c r="N18" t="n">
-        <v>10997624</v>
+        <v>196783125</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>10997624</v>
+        <v>196783125</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -4621,56 +4627,50 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>22-09-2026</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.062</v>
+        <v>2.831</v>
       </c>
       <c r="W18" t="n">
-        <v>1782</v>
+        <v>695</v>
       </c>
       <c r="X18" t="n">
-        <v>40.9</v>
+        <v>26.1</v>
       </c>
       <c r="Y18" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Z18" t="n">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="AA18" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.8</v>
+        <v>7.88</v>
       </c>
       <c r="AC18" t="n">
-        <v>30.3</v>
+        <v>14.1</v>
       </c>
       <c r="AD18" t="n">
-        <v>0.2</v>
+        <v>0.32</v>
       </c>
       <c r="AE18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF18" t="n">
-        <v>23</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>178.38</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>487.24</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>29.5</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
       <c r="AJ18" t="n">
-        <v>171.837875</v>
+        <v>143.7164139971926</v>
       </c>
       <c r="AK18" t="n">
-        <v>-18.2</v>
+        <v>-0.9</v>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
@@ -4689,31 +4689,31 @@
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>22-09-2026</t>
         </is>
       </c>
       <c r="AQ18" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="AR18" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="AS18" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="AT18" t="n">
         <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AW18" t="n">
         <v>4</v>
@@ -4725,16 +4725,16 @@
         <v>0</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0</v>
+        <v>196783125</v>
       </c>
       <c r="BA18" t="n">
-        <v>6076769</v>
+        <v>196783125</v>
       </c>
       <c r="BB18" t="n">
-        <v>10997624</v>
+        <v>196783125</v>
       </c>
       <c r="BC18" t="n">
-        <v>10997624</v>
+        <v>196783125</v>
       </c>
       <c r="BD18" t="n">
         <v>0</v>
@@ -4770,7 +4770,7 @@
         <v>0</v>
       </c>
       <c r="BO18" t="n">
-        <v>6076769</v>
+        <v>196783125</v>
       </c>
       <c r="BP18" t="n">
         <v>1</v>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.321</v>
+        <v>0.316</v>
       </c>
       <c r="W19" t="n">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="X19" t="n">
-        <v>23.9</v>
+        <v>24.2</v>
       </c>
       <c r="Y19" t="n">
         <v>12</v>
@@ -5089,13 +5089,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.374</v>
+        <v>0.375</v>
       </c>
       <c r="W20" t="n">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="X20" t="n">
-        <v>53.6</v>
+        <v>53.5</v>
       </c>
       <c r="Y20" t="n">
         <v>21</v>
@@ -5321,13 +5321,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.649</v>
+        <v>0.651</v>
       </c>
       <c r="W21" t="n">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="X21" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="Y21" t="n">
         <v>19</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="W22" t="n">
-        <v>670</v>
+        <v>651</v>
       </c>
       <c r="X22" t="n">
-        <v>10.9</v>
+        <v>10.6</v>
       </c>
       <c r="Y22" t="n">
         <v>-5</v>
@@ -5788,10 +5788,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W23" t="n">
-        <v>53106</v>
+        <v>52727</v>
       </c>
       <c r="X23" t="n">
-        <v>45</v>
+        <v>44.6</v>
       </c>
       <c r="Y23" t="n">
         <v>5</v>
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.183</v>
+        <v>0.184</v>
       </c>
       <c r="W24" t="n">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="X24" t="n">
-        <v>50.7</v>
+        <v>50.4</v>
       </c>
       <c r="Y24" t="n">
         <v>3</v>
@@ -6041,7 +6041,7 @@
         <v>11.6</v>
       </c>
       <c r="AD24" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE24" t="b">
         <v>1</v>
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.927</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="W25" t="n">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="X25" t="n">
-        <v>6.27</v>
+        <v>6.16</v>
       </c>
       <c r="Y25" t="n">
         <v>31</v>
@@ -6477,13 +6477,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.643</v>
+        <v>0.633</v>
       </c>
       <c r="W26" t="n">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="X26" t="n">
-        <v>1178</v>
+        <v>1197</v>
       </c>
       <c r="Y26" t="n">
         <v>-61</v>
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>1.876</v>
+        <v>1.926</v>
       </c>
       <c r="W27" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="n">
@@ -6935,13 +6935,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.274</v>
+        <v>0.276</v>
       </c>
       <c r="W28" t="n">
-        <v>950</v>
+        <v>942</v>
       </c>
       <c r="X28" t="n">
-        <v>25.9</v>
+        <v>25.6</v>
       </c>
       <c r="Y28" t="n">
         <v>9</v>
@@ -7167,13 +7167,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.495</v>
+        <v>0.5</v>
       </c>
       <c r="W29" t="n">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="X29" t="n">
-        <v>37.6</v>
+        <v>37.2</v>
       </c>
       <c r="Y29" t="n">
         <v>-44</v>
@@ -7399,13 +7399,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.199</v>
+        <v>0.204</v>
       </c>
       <c r="W30" t="n">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="X30" t="n">
-        <v>14.6</v>
+        <v>14.4</v>
       </c>
       <c r="Y30" t="n">
         <v>16</v>
@@ -7860,10 +7860,10 @@
         <v>0.045</v>
       </c>
       <c r="W32" t="n">
-        <v>1550</v>
+        <v>1553</v>
       </c>
       <c r="X32" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="Y32" t="n">
         <v>10</v>
@@ -8092,7 +8092,7 @@
         <v>0.229</v>
       </c>
       <c r="W33" t="n">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="X33" t="n">
         <v>13.5</v>
@@ -8321,13 +8321,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.786</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="W34" t="n">
-        <v>4019</v>
+        <v>3903</v>
       </c>
       <c r="X34" t="n">
-        <v>28.1</v>
+        <v>27.3</v>
       </c>
       <c r="Y34" t="n">
         <v>2</v>
@@ -8553,13 +8553,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.23</v>
+        <v>0.227</v>
       </c>
       <c r="W35" t="n">
-        <v>1734</v>
+        <v>1758</v>
       </c>
       <c r="X35" t="n">
-        <v>18.3</v>
+        <v>18.6</v>
       </c>
       <c r="Y35" t="n">
         <v>-3</v>
@@ -8785,13 +8785,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.359</v>
+        <v>0.363</v>
       </c>
       <c r="W36" t="n">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="X36" t="n">
-        <v>96.59999999999999</v>
+        <v>95.7</v>
       </c>
       <c r="Y36" t="n">
         <v>246</v>
@@ -9017,13 +9017,13 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="W37" t="n">
-        <v>9884</v>
+        <v>9515</v>
       </c>
       <c r="X37" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="Y37" t="n">
         <v>-12</v>
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="V38" t="n">
-        <v>0.04</v>
+        <v>0.041</v>
       </c>
       <c r="W38" t="n">
-        <v>3328</v>
+        <v>3310</v>
       </c>
       <c r="X38" t="n">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="Y38" t="n">
         <v>-4</v>
@@ -9484,7 +9484,7 @@
         <v>0.011</v>
       </c>
       <c r="W39" t="n">
-        <v>4163</v>
+        <v>4127</v>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="n">
@@ -9714,10 +9714,10 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>4928</v>
+        <v>4932</v>
       </c>
       <c r="X40" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="Y40" t="n">
         <v>26</v>
@@ -9943,13 +9943,13 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0.104</v>
+        <v>0.106</v>
       </c>
       <c r="W41" t="n">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="X41" t="n">
-        <v>26.3</v>
+        <v>25.8</v>
       </c>
       <c r="Y41" t="n">
         <v>24</v>
@@ -10175,13 +10175,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.12</v>
+        <v>0.114</v>
       </c>
       <c r="W42" t="n">
-        <v>415</v>
+        <v>437</v>
       </c>
       <c r="X42" t="n">
-        <v>6.7</v>
+        <v>7.09</v>
       </c>
       <c r="Y42" t="n">
         <v>118</v>
@@ -10331,16 +10331,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -10348,40 +10348,40 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
-        <v>15</v>
+        <v>-5</v>
       </c>
       <c r="G43" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>389.15</v>
+        <v>666.2</v>
       </c>
       <c r="J43" t="n">
-        <v>338.1</v>
+        <v>622.4400000000001</v>
       </c>
       <c r="K43" t="n">
-        <v>15.1</v>
+        <v>7</v>
       </c>
       <c r="L43" t="n">
-        <v>66.73</v>
+        <v>74.02</v>
       </c>
       <c r="M43" t="n">
-        <v>0.34</v>
+        <v>0.49</v>
       </c>
       <c r="N43" t="n">
-        <v>3381000</v>
+        <v>4930931</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>3381000</v>
+        <v>4930931</v>
       </c>
       <c r="Q43" t="n">
         <v>0</v>
@@ -10395,124 +10395,122 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.074</v>
+        <v>0.05</v>
       </c>
       <c r="W43" t="n">
-        <v>459</v>
-      </c>
-      <c r="X43" t="n">
-        <v>13.6</v>
-      </c>
+        <v>983</v>
+      </c>
+      <c r="X43" t="inlineStr"/>
       <c r="Y43" t="n">
-        <v>-8</v>
+        <v>-2</v>
       </c>
       <c r="Z43" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="AA43" t="n">
-        <v>33</v>
+        <v>-152</v>
       </c>
       <c r="AB43" t="n">
-        <v>14.36</v>
+        <v>-6.5</v>
       </c>
       <c r="AC43" t="n">
-        <v>9.94</v>
+        <v>9.24</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.23</v>
+        <v>2.23</v>
       </c>
       <c r="AE43" t="b">
         <v>1</v>
       </c>
       <c r="AF43" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="AG43" t="n">
-        <v>366.73</v>
+        <v>598.4</v>
       </c>
       <c r="AH43" t="n">
-        <v>272.07</v>
+        <v>549.58</v>
       </c>
       <c r="AI43" t="n">
-        <v>99.5</v>
+        <v>36.6</v>
       </c>
       <c r="AJ43" t="n">
-        <v>338.1</v>
+        <v>622.4351173945973</v>
       </c>
       <c r="AK43" t="n">
-        <v>15.1</v>
+        <v>7</v>
       </c>
       <c r="AL43" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM43" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN43" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="AQ43" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="AR43" t="n">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="AS43" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AT43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV43" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AX43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AY43" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="AZ43" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="BA43" t="n">
-        <v>0</v>
+        <v>3760931</v>
       </c>
       <c r="BB43" t="n">
-        <v>3381000</v>
+        <v>4930931</v>
       </c>
       <c r="BC43" t="n">
-        <v>3381000</v>
+        <v>4930931</v>
       </c>
       <c r="BD43" t="n">
         <v>0</v>
@@ -10545,34 +10543,34 @@
         <v>0</v>
       </c>
       <c r="BN43" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="BO43" t="n">
-        <v>0</v>
+        <v>3760931</v>
       </c>
       <c r="BP43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ43" t="n">
         <v>0</v>
       </c>
       <c r="BR43" t="n">
-        <v>0</v>
+        <v>0.6575</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -10580,40 +10578,40 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G44" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>35.05</v>
+        <v>389.15</v>
       </c>
       <c r="J44" t="n">
-        <v>23.55</v>
+        <v>338.1</v>
       </c>
       <c r="K44" t="n">
-        <v>48.8</v>
+        <v>15.1</v>
       </c>
       <c r="L44" t="n">
-        <v>68.34</v>
+        <v>66.73</v>
       </c>
       <c r="M44" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="N44" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="Q44" t="n">
         <v>0</v>
@@ -10627,124 +10625,124 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.113</v>
+        <v>0.075</v>
       </c>
       <c r="W44" t="n">
-        <v>179</v>
+        <v>450</v>
       </c>
       <c r="X44" t="n">
-        <v>41.4</v>
+        <v>13.3</v>
       </c>
       <c r="Y44" t="n">
-        <v>19</v>
+        <v>-8</v>
       </c>
       <c r="Z44" t="n">
-        <v>3.17</v>
+        <v>24</v>
       </c>
       <c r="AA44" t="n">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.49</v>
+        <v>14.36</v>
       </c>
       <c r="AC44" t="n">
-        <v>8.76</v>
+        <v>9.94</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="AE44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF44" t="n">
-        <v>14.87</v>
+        <v>18</v>
       </c>
       <c r="AG44" t="n">
-        <v>23.74</v>
+        <v>366.73</v>
       </c>
       <c r="AH44" t="n">
-        <v>22.79</v>
+        <v>272.07</v>
       </c>
       <c r="AI44" t="n">
-        <v>92.8</v>
+        <v>99.5</v>
       </c>
       <c r="AJ44" t="n">
-        <v>23.5472893358377</v>
+        <v>338.1</v>
       </c>
       <c r="AK44" t="n">
-        <v>48.8</v>
+        <v>15.1</v>
       </c>
       <c r="AL44" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM44" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN44" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO44" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AQ44" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="AR44" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="AS44" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="AT44" t="n">
         <v>0</v>
       </c>
       <c r="AU44" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AV44" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AW44" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AX44" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AY44" t="n">
         <v>0</v>
       </c>
       <c r="AZ44" t="n">
-        <v>1188529</v>
+        <v>0</v>
       </c>
       <c r="BA44" t="n">
-        <v>1457700</v>
+        <v>0</v>
       </c>
       <c r="BB44" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="BC44" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="BD44" t="n">
         <v>0</v>
@@ -10780,10 +10778,10 @@
         <v>0</v>
       </c>
       <c r="BO44" t="n">
-        <v>1457700</v>
+        <v>0</v>
       </c>
       <c r="BP44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BQ44" t="n">
         <v>0</v>
@@ -10795,16 +10793,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -10812,10 +10810,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
-        <v>-5</v>
+        <v>4</v>
       </c>
       <c r="G45" t="n">
         <v>25</v>
@@ -10824,28 +10822,28 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>666.2</v>
+        <v>35.05</v>
       </c>
       <c r="J45" t="n">
-        <v>593.62</v>
+        <v>23.55</v>
       </c>
       <c r="K45" t="n">
-        <v>12.2</v>
+        <v>48.8</v>
       </c>
       <c r="L45" t="n">
-        <v>74.02</v>
+        <v>68.34</v>
       </c>
       <c r="M45" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="N45" t="n">
-        <v>2458195</v>
+        <v>2018403</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>2458195</v>
+        <v>2018403</v>
       </c>
       <c r="Q45" t="n">
         <v>0</v>
@@ -10859,58 +10857,60 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.024</v>
+        <v>0.119</v>
       </c>
       <c r="W45" t="n">
-        <v>1035</v>
-      </c>
-      <c r="X45" t="inlineStr"/>
+        <v>170</v>
+      </c>
+      <c r="X45" t="n">
+        <v>39.4</v>
+      </c>
       <c r="Y45" t="n">
-        <v>-2</v>
+        <v>19</v>
       </c>
       <c r="Z45" t="n">
-        <v>5</v>
+        <v>3.17</v>
       </c>
       <c r="AA45" t="n">
-        <v>-152</v>
+        <v>7</v>
       </c>
       <c r="AB45" t="n">
-        <v>-6.5</v>
+        <v>0.49</v>
       </c>
       <c r="AC45" t="n">
-        <v>9.24</v>
+        <v>8.76</v>
       </c>
       <c r="AD45" t="n">
-        <v>2.23</v>
+        <v>0.2</v>
       </c>
       <c r="AE45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF45" t="n">
-        <v>6</v>
+        <v>14.87</v>
       </c>
       <c r="AG45" t="n">
-        <v>598.4</v>
+        <v>23.74</v>
       </c>
       <c r="AH45" t="n">
-        <v>549.58</v>
+        <v>22.79</v>
       </c>
       <c r="AI45" t="n">
-        <v>36.6</v>
+        <v>92.8</v>
       </c>
       <c r="AJ45" t="n">
-        <v>593.6235208886742</v>
+        <v>23.5472893358377</v>
       </c>
       <c r="AK45" t="n">
-        <v>12.2</v>
+        <v>48.8</v>
       </c>
       <c r="AL45" t="inlineStr">
         <is>
@@ -10924,57 +10924,57 @@
       </c>
       <c r="AN45" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO45" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="AQ45" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="AR45" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="AS45" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="AT45" t="n">
         <v>0</v>
       </c>
       <c r="AU45" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AV45" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="AW45" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="AX45" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="AY45" t="n">
         <v>0</v>
       </c>
       <c r="AZ45" t="n">
-        <v>0</v>
+        <v>1188529</v>
       </c>
       <c r="BA45" t="n">
-        <v>1288195</v>
+        <v>1457700</v>
       </c>
       <c r="BB45" t="n">
-        <v>2458195</v>
+        <v>2018403</v>
       </c>
       <c r="BC45" t="n">
-        <v>2458195</v>
+        <v>2018403</v>
       </c>
       <c r="BD45" t="n">
         <v>0</v>
@@ -11010,10 +11010,10 @@
         <v>0</v>
       </c>
       <c r="BO45" t="n">
-        <v>1288195</v>
+        <v>1457700</v>
       </c>
       <c r="BP45" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="BQ45" t="n">
         <v>0</v>
@@ -11100,10 +11100,10 @@
         <v>0.008</v>
       </c>
       <c r="W46" t="n">
-        <v>5260</v>
+        <v>5212</v>
       </c>
       <c r="X46" t="n">
-        <v>8.890000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="Y46" t="n">
         <v>43</v>
@@ -11329,13 +11329,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="W47" t="n">
-        <v>5130</v>
+        <v>4936</v>
       </c>
       <c r="X47" t="n">
-        <v>13.2</v>
+        <v>12.7</v>
       </c>
       <c r="Y47" t="n">
         <v>23</v>
@@ -11560,10 +11560,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>8856</v>
+        <v>8769</v>
       </c>
       <c r="X48" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
@@ -11789,13 +11789,13 @@
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.211</v>
+        <v>0.213</v>
       </c>
       <c r="W49" t="n">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="X49" t="n">
-        <v>25.3</v>
+        <v>25.1</v>
       </c>
       <c r="Y49" t="n">
         <v>21</v>
@@ -12024,10 +12024,10 @@
         <v>0</v>
       </c>
       <c r="W50" t="n">
-        <v>3682</v>
+        <v>3690</v>
       </c>
       <c r="X50" t="n">
-        <v>82.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="Y50" t="n">
         <v>42</v>
@@ -12256,10 +12256,10 @@
         <v>0</v>
       </c>
       <c r="W51" t="n">
-        <v>115770</v>
+        <v>113842</v>
       </c>
       <c r="X51" t="n">
-        <v>33.3</v>
+        <v>32.7</v>
       </c>
       <c r="Y51" t="n">
         <v>18</v>
@@ -12765,245 +12765,245 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>68.59999999999999</v>
+        <v>1043.35</v>
       </c>
       <c r="D10" t="n">
-        <v>64.48999999999999</v>
+        <v>799.34</v>
       </c>
       <c r="E10" t="n">
-        <v>6.4</v>
+        <v>30.5</v>
       </c>
       <c r="F10" t="n">
-        <v>64.29000000000001</v>
+        <v>61.71</v>
       </c>
       <c r="G10" t="n">
-        <v>0.57</v>
+        <v>3.2</v>
       </c>
       <c r="H10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>28-09-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5062</v>
+        <v>140.49</v>
       </c>
       <c r="D11" t="n">
-        <v>5198.76</v>
+        <v>171.54</v>
       </c>
       <c r="E11" t="n">
-        <v>-2.6</v>
+        <v>-18.1</v>
       </c>
       <c r="F11" t="n">
-        <v>67.16</v>
+        <v>74.59</v>
       </c>
       <c r="G11" t="n">
-        <v>7.21</v>
+        <v>1.11</v>
       </c>
       <c r="H11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1043.35</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>799.34</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>30.5</v>
+        <v>6.4</v>
       </c>
       <c r="F12" t="n">
-        <v>61.71</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>3.2</v>
+        <v>0.57</v>
       </c>
       <c r="H12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>28-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hy-Tech Engineers Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>72.29000000000001</v>
+        <v>5062</v>
       </c>
       <c r="D13" t="n">
-        <v>68.68000000000001</v>
+        <v>5198.76</v>
       </c>
       <c r="E13" t="n">
-        <v>5.3</v>
+        <v>-2.6</v>
       </c>
       <c r="F13" t="n">
-        <v>71.22</v>
+        <v>67.16</v>
       </c>
       <c r="G13" t="n">
-        <v>0.86</v>
+        <v>7.21</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bhageria Industries Limited</t>
+          <t>Hy-Tech Engineers Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>406.45</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>217.8</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>86.59999999999999</v>
+        <v>5.3</v>
       </c>
       <c r="F14" t="n">
-        <v>71.75</v>
+        <v>71.22</v>
       </c>
       <c r="G14" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INDO RAMA SYNTHETICS (INDIA) LIMITED</t>
+          <t>Bhageria Industries Limited</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>100.36</v>
+        <v>406.45</v>
       </c>
       <c r="D15" t="n">
-        <v>75.68000000000001</v>
+        <v>217.8</v>
       </c>
       <c r="E15" t="n">
-        <v>32.6</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>74.84999999999999</v>
+        <v>71.75</v>
       </c>
       <c r="G15" t="n">
-        <v>3.14</v>
+        <v>0.82</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VEEGALAND</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>INDO RAMA SYNTHETICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>142.41</v>
+        <v>100.36</v>
       </c>
       <c r="D16" t="n">
-        <v>143.72</v>
+        <v>75.68000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.9</v>
+        <v>32.6</v>
       </c>
       <c r="F16" t="n">
-        <v>63.69</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>19.68</v>
+        <v>3.14</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>22-09-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
     </row>
@@ -13045,35 +13045,35 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>VEEGALAND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>140.49</v>
+        <v>142.41</v>
       </c>
       <c r="D18" t="n">
-        <v>171.84</v>
+        <v>143.72</v>
       </c>
       <c r="E18" t="n">
-        <v>-18.2</v>
+        <v>-0.9</v>
       </c>
       <c r="F18" t="n">
-        <v>74.59</v>
+        <v>63.69</v>
       </c>
       <c r="G18" t="n">
-        <v>1.1</v>
+        <v>19.68</v>
       </c>
       <c r="H18" t="n">
         <v>4</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>22-09-2026</t>
         </is>
       </c>
     </row>
@@ -13920,105 +13920,105 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>389.15</v>
+        <v>666.2</v>
       </c>
       <c r="D43" t="n">
-        <v>338.1</v>
+        <v>622.4400000000001</v>
       </c>
       <c r="E43" t="n">
-        <v>15.1</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
-        <v>66.73</v>
+        <v>74.02</v>
       </c>
       <c r="G43" t="n">
-        <v>0.34</v>
+        <v>0.49</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>35.05</v>
+        <v>389.15</v>
       </c>
       <c r="D44" t="n">
-        <v>23.55</v>
+        <v>338.1</v>
       </c>
       <c r="E44" t="n">
-        <v>48.8</v>
+        <v>15.1</v>
       </c>
       <c r="F44" t="n">
-        <v>68.34</v>
+        <v>66.73</v>
       </c>
       <c r="G44" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="H44" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>666.2</v>
+        <v>35.05</v>
       </c>
       <c r="D45" t="n">
-        <v>593.62</v>
+        <v>23.55</v>
       </c>
       <c r="E45" t="n">
-        <v>12.2</v>
+        <v>48.8</v>
       </c>
       <c r="F45" t="n">
-        <v>74.02</v>
+        <v>68.34</v>
       </c>
       <c r="G45" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
@@ -14265,7 +14265,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -14275,7 +14275,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -14315,7 +14315,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -14335,7 +14335,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">

</xml_diff>